<commit_message>
Update: tooltips, workflow schedule, and budget logic refinements
</commit_message>
<xml_diff>
--- a/main/reca.xlsx
+++ b/main/reca.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ivanrodriguez/Documents/Antigravity/Coparticipacion/main/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{989599A1-F914-B042-9414-A97C562A2A81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{434EDA9C-A846-6F40-AA2A-3A567612921A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38400" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{E327F0F6-7896-FA43-9329-53B85594D54E}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="21000" xr2:uid="{E327F0F6-7896-FA43-9329-53B85594D54E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -442,7 +442,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A42FF238-21C6-E649-9163-1DB4C100D5AC}">
-  <dimension ref="A1:J27"/>
+  <dimension ref="A1:Q30"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="15.5" bestFit="1" customWidth="1"/>
@@ -842,19 +842,19 @@
         <v>132982541.30000001</v>
       </c>
       <c r="D14" s="1">
-        <v>0</v>
+        <v>301332387.03999996</v>
       </c>
       <c r="E14" s="1">
-        <v>0</v>
+        <v>26222347.5</v>
       </c>
       <c r="F14" s="1">
-        <v>3946414459.4400005</v>
+        <v>3946414459.4400001</v>
       </c>
       <c r="G14" s="1">
         <v>38879706.869999997</v>
       </c>
       <c r="H14" s="1">
-        <v>24616070000</v>
+        <v>24616070257.452999</v>
       </c>
       <c r="I14" s="1">
         <v>0</v>
@@ -871,19 +871,19 @@
         <v>231174736.18000001</v>
       </c>
       <c r="D15" s="1">
-        <v>0</v>
+        <v>271067467.48000002</v>
       </c>
       <c r="E15" s="1">
-        <v>0</v>
+        <v>33395905.169999998</v>
       </c>
       <c r="F15" s="1">
-        <v>3861033580.8700008</v>
+        <v>3861033580.8699999</v>
       </c>
       <c r="G15" s="1">
         <v>39521711.210000001</v>
       </c>
       <c r="H15" s="1">
-        <v>24407000000</v>
+        <v>24406996560.783001</v>
       </c>
       <c r="I15" s="1">
         <v>0</v>
@@ -900,25 +900,25 @@
         <v>343764424.43000001</v>
       </c>
       <c r="D16" s="1">
-        <v>0</v>
+        <v>454061717.14999998</v>
       </c>
       <c r="E16" s="1">
-        <v>0</v>
+        <v>42600930.340000004</v>
       </c>
       <c r="F16" s="1">
-        <v>4051880463.4800005</v>
+        <v>4051880463.48</v>
       </c>
       <c r="G16" s="1">
         <v>35184779.129999995</v>
       </c>
       <c r="H16" s="1">
-        <v>23487050000</v>
+        <v>23487046606.860001</v>
       </c>
       <c r="I16" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A17">
         <v>2025</v>
       </c>
@@ -929,10 +929,10 @@
         <v>3381349416.96</v>
       </c>
       <c r="D17" s="1">
-        <v>0</v>
+        <v>348733642.34999996</v>
       </c>
       <c r="E17" s="1">
-        <v>0</v>
+        <v>40025270.660000004</v>
       </c>
       <c r="F17" s="1">
         <v>4285413146.77</v>
@@ -941,13 +941,13 @@
         <v>51226082.25</v>
       </c>
       <c r="H17" s="1">
-        <v>24338750000</v>
+        <v>24338754124.333004</v>
       </c>
       <c r="I17" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A18">
         <v>2025</v>
       </c>
@@ -955,16 +955,16 @@
         <v>5</v>
       </c>
       <c r="C18" s="1">
-        <v>429720806.67999995</v>
+        <v>429720806.67999989</v>
       </c>
       <c r="D18" s="1">
-        <v>0</v>
+        <v>286999162.62</v>
       </c>
       <c r="E18" s="1">
-        <v>0</v>
+        <v>38861728.25</v>
       </c>
       <c r="F18" s="1">
-        <v>4028167357.5399995</v>
+        <v>4028167357.54</v>
       </c>
       <c r="G18" s="1">
         <v>40746668.230000004</v>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A19">
         <v>2025</v>
       </c>
@@ -987,10 +987,10 @@
         <v>1145641669.6699996</v>
       </c>
       <c r="D19" s="1">
-        <v>0</v>
+        <v>268540705.16000009</v>
       </c>
       <c r="E19" s="1">
-        <v>0</v>
+        <v>47238047.540000007</v>
       </c>
       <c r="F19" s="1">
         <v>4640691232.5900002</v>
@@ -999,13 +999,13 @@
         <v>47771828.409999996</v>
       </c>
       <c r="H19" s="1">
-        <v>25520330000</v>
+        <v>25520330123.800007</v>
       </c>
       <c r="I19" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A20">
         <v>2025</v>
       </c>
@@ -1016,25 +1016,25 @@
         <v>443956265.43000007</v>
       </c>
       <c r="D20" s="1">
-        <v>0</v>
+        <v>339809028.70999998</v>
       </c>
       <c r="E20" s="1">
-        <v>0</v>
+        <v>28389994.539999999</v>
       </c>
       <c r="F20" s="1">
-        <v>4329250661.0599995</v>
+        <v>4329250661.0600004</v>
       </c>
       <c r="G20" s="1">
         <v>54193716.850000001</v>
       </c>
       <c r="H20" s="1">
-        <v>26235900000</v>
+        <v>26235896387.789997</v>
       </c>
       <c r="I20" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A21">
         <v>2025</v>
       </c>
@@ -1045,13 +1045,13 @@
         <v>1079600954.6699998</v>
       </c>
       <c r="D21" s="1">
-        <v>0</v>
+        <v>311493623.15000015</v>
       </c>
       <c r="E21" s="1">
-        <v>0</v>
+        <v>23953286.25</v>
       </c>
       <c r="F21" s="1">
-        <v>4999874909.6999989</v>
+        <v>4999874909.6999998</v>
       </c>
       <c r="G21" s="1">
         <v>64351329.269999996</v>
@@ -1063,7 +1063,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A22">
         <v>2025</v>
       </c>
@@ -1074,13 +1074,13 @@
         <v>595274035.79999995</v>
       </c>
       <c r="D22" s="1">
-        <v>0</v>
+        <v>306077501.50999999</v>
       </c>
       <c r="E22" s="1">
-        <v>0</v>
+        <v>24112253.050000001</v>
       </c>
       <c r="F22" s="1">
-        <v>4988757388.4800005</v>
+        <v>4988757388.4799995</v>
       </c>
       <c r="G22" s="1">
         <v>49692085.07</v>
@@ -1092,7 +1092,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A23">
         <v>2025</v>
       </c>
@@ -1103,25 +1103,25 @@
         <v>1145329731.76</v>
       </c>
       <c r="D23" s="1">
-        <v>0</v>
+        <v>257327566.68999997</v>
       </c>
       <c r="E23" s="1">
-        <v>0</v>
+        <v>23862068.759999998</v>
       </c>
       <c r="F23" s="1">
-        <v>4480525230.2200022</v>
+        <v>4480525230.2200003</v>
       </c>
       <c r="G23" s="1">
         <v>50164545.629999995</v>
       </c>
       <c r="H23" s="1">
-        <v>27963350345.420002</v>
+        <v>27963353246.540001</v>
       </c>
       <c r="I23" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A24">
         <v>2025</v>
       </c>
@@ -1132,25 +1132,25 @@
         <v>509264678.54000008</v>
       </c>
       <c r="D24" s="1">
-        <v>0</v>
+        <v>227838596.24000001</v>
       </c>
       <c r="E24" s="1">
-        <v>0</v>
+        <v>33800092.740000002</v>
       </c>
       <c r="F24" s="1">
-        <v>3985854751.249999</v>
+        <v>3985854751.25</v>
       </c>
       <c r="G24" s="1">
         <v>35773379.289999999</v>
       </c>
       <c r="H24" s="1">
-        <v>27718065527.080002</v>
+        <v>27718069339.25</v>
       </c>
       <c r="I24" s="1">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A25">
         <v>2025</v>
       </c>
@@ -1161,10 +1161,10 @@
         <v>279456392.82999998</v>
       </c>
       <c r="D25" s="1">
-        <v>0</v>
+        <v>300524147.13</v>
       </c>
       <c r="E25" s="1">
-        <v>0</v>
+        <v>34722570.450000003</v>
       </c>
       <c r="F25" s="1">
         <v>4265353849.5100002</v>
@@ -1173,14 +1173,14 @@
         <v>64239524.140000001</v>
       </c>
       <c r="H25" s="1">
-        <v>28412888136.260002</v>
+        <v>28412888136.259998</v>
       </c>
       <c r="I25" s="1">
         <v>0</v>
       </c>
       <c r="J25" s="1"/>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A26">
         <v>2026</v>
       </c>
@@ -1210,7 +1210,7 @@
       </c>
       <c r="J26" s="1"/>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A27">
         <v>2026</v>
       </c>
@@ -1239,6 +1239,20 @@
         <v>37413.79</v>
       </c>
       <c r="J27" s="1"/>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.2">
+      <c r="F30" s="1"/>
+      <c r="G30" s="1"/>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
+      <c r="K30" s="1"/>
+      <c r="L30" s="1"/>
+      <c r="M30" s="1"/>
+      <c r="N30" s="1"/>
+      <c r="O30" s="1"/>
+      <c r="P30" s="1"/>
+      <c r="Q30" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>